<commit_message>
game: give every starter companion a manual ability
Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/Assets/@Resources/Data/Excel/LocalizationData.xlsx
+++ b/Assets/@Resources/Data/Excel/LocalizationData.xlsx
@@ -2271,7 +2271,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>당신는(은) 매력발산!를(을) 사용했다!</t>
+          <t>매력을 발산해 미니몬의 관심을 끌었다!</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -4920,12 +4920,18 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>젤리 퐁의 고유기술. 최대 체력을 늘린다.</t>
+          <t>기본 효과: 단계당 최대 체력 +30.
+수동 사용: 최대 체력의 18% × 능력 단계만큼 회복한다.
+재사용 18초(미니몬 능력끼리 공유).
+동행 중 임시 사용 가능. 공명도 100%에서 영구 습득.</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Jelly Pong's unique skill. Increases max HP.</t>
+          <t>Passive: +30 maximum HP per ability level.
+Manual use: Restore 18% of maximum HP per ability level.
+Cooldown: 18s, shared by minion abilities.
+Available temporarily while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
     </row>
@@ -4973,12 +4979,18 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>라비 슬라임의 고유기술. 공격속도를 높인다.</t>
+          <t>기본 효과: 단계당 공격속도 +10%p.
+수동 사용: 8초 동안 공격속도가 30%p × 능력 단계만큼 오른다.
+재사용 18초(미니몬 능력끼리 공유).
+동행 중 임시 사용 가능. 공명도 100%에서 영구 습득.</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Rabi Slime's unique skill. Increases attack speed.</t>
+          <t>Passive: +10 percentage points of attack speed per ability level.
+Manual use: Gain 30 percentage points of attack speed per ability level for 8 seconds.
+Cooldown: 18s, shared by minion abilities.
+Available temporarily while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
game: make combat abilities visible and readable
Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/Assets/@Resources/Data/Excel/LocalizationData.xlsx
+++ b/Assets/@Resources/Data/Excel/LocalizationData.xlsx
@@ -328,7 +328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1840"/>
+  <dimension ref="A1:C1845"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -33797,6 +33797,91 @@
         </is>
       </c>
     </row>
+    <row r="1841">
+      <c r="A1841" t="inlineStr">
+        <is>
+          <t>CombatAbilityReadyText</t>
+        </is>
+      </c>
+      <c r="B1841" t="inlineStr">
+        <is>
+          <t>눌러서 사용</t>
+        </is>
+      </c>
+      <c r="C1841" t="inlineStr">
+        <is>
+          <t>Tap to use</t>
+        </is>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" t="inlineStr">
+        <is>
+          <t>CombatAbilityCooldownText</t>
+        </is>
+      </c>
+      <c r="B1842" t="inlineStr">
+        <is>
+          <t>재사용 대기</t>
+        </is>
+      </c>
+      <c r="C1842" t="inlineStr">
+        <is>
+          <t>Cooling down</t>
+        </is>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" t="inlineStr">
+        <is>
+          <t>CombatAbilityFullHpText</t>
+        </is>
+      </c>
+      <c r="B1843" t="inlineStr">
+        <is>
+          <t>체력이 가득합니다</t>
+        </is>
+      </c>
+      <c r="C1843" t="inlineStr">
+        <is>
+          <t>Health is full</t>
+        </is>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" t="inlineStr">
+        <is>
+          <t>CombatAbilityNoTargetText</t>
+        </is>
+      </c>
+      <c r="B1844" t="inlineStr">
+        <is>
+          <t>적을 기다리는 중</t>
+        </is>
+      </c>
+      <c r="C1844" t="inlineStr">
+        <is>
+          <t>Waiting for a target</t>
+        </is>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" t="inlineStr">
+        <is>
+          <t>CombatAbilityUnavailableText</t>
+        </is>
+      </c>
+      <c r="B1845" t="inlineStr">
+        <is>
+          <t>지금은 사용할 수 없습니다</t>
+        </is>
+      </c>
+      <c r="C1845" t="inlineStr">
+        <is>
+          <t>Unavailable</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
game: make class choices distinct and show their actual effects
Co-Authored-By: Codex <noreply@openai.com>
</commit_message>
<xml_diff>
--- a/Assets/@Resources/Data/Excel/LocalizationData.xlsx
+++ b/Assets/@Resources/Data/Excel/LocalizationData.xlsx
@@ -328,7 +328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1851"/>
+  <dimension ref="A1:C1878"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4765,12 +4765,12 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>최대 체력을 증가시킨다.</t>
+          <t>최대 체력과 방어력이 오른다.</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Increases max HP.</t>
+          <t>Increases max HP and defense.</t>
         </is>
       </c>
     </row>
@@ -5092,7 +5092,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Physical attack rises for a while at battle start.</t>
+          <t>Increases physical attack briefly when entering a battle area.</t>
         </is>
       </c>
     </row>
@@ -15576,7 +15576,7 @@
       </c>
       <c r="C887" t="inlineStr">
         <is>
-          <t>선제의 감각</t>
+          <t>First Strike Instinct</t>
         </is>
       </c>
     </row>
@@ -15593,7 +15593,7 @@
       </c>
       <c r="C888" t="inlineStr">
         <is>
-          <t>전투 시작 시 60% 확률로 공격력이 잠시 오른다</t>
+          <t>A 60% chance to briefly increase physical attack when entering a battle area.</t>
         </is>
       </c>
     </row>
@@ -15746,7 +15746,7 @@
       </c>
       <c r="C897" t="inlineStr">
         <is>
-          <t>연쇄 각성</t>
+          <t>Chain Awakening</t>
         </is>
       </c>
     </row>
@@ -15763,7 +15763,7 @@
       </c>
       <c r="C898" t="inlineStr">
         <is>
-          <t>연속 3회 치명타 시 큰 피해를 추가한다</t>
+          <t>Deals bonus damage after three consecutive critical hits.</t>
         </is>
       </c>
     </row>
@@ -15882,7 +15882,7 @@
       </c>
       <c r="C905" t="inlineStr">
         <is>
-          <t>그림자 걸음</t>
+          <t>Shadow Step</t>
         </is>
       </c>
     </row>
@@ -15899,7 +15899,7 @@
       </c>
       <c r="C906" t="inlineStr">
         <is>
-          <t>연속 3회 회피 시 회피율이 크게 오른다</t>
+          <t>Briefly increases evasion after three consecutive dodges.</t>
         </is>
       </c>
     </row>
@@ -16018,7 +16018,7 @@
       </c>
       <c r="C913" t="inlineStr">
         <is>
-          <t>불굴</t>
+          <t>Indomitable</t>
         </is>
       </c>
     </row>
@@ -16030,12 +16030,12 @@
       </c>
       <c r="B914" t="inlineStr">
         <is>
-          <t>치명상을 입을 때 40% 확률로 체력을 회복하며 버틴다</t>
+          <t>치명 피해를 받기 직전 40% 확률로 체력을 회복한다.</t>
         </is>
       </c>
       <c r="C914" t="inlineStr">
         <is>
-          <t>치명상을 입을 때 40% 확률로 체력을 회복하며 버틴다</t>
+          <t>A 40% chance to restore HP just before taking an otherwise fatal hit.</t>
         </is>
       </c>
     </row>
@@ -16120,7 +16120,7 @@
       </c>
       <c r="C919" t="inlineStr">
         <is>
-          <t>각성</t>
+          <t>Awakening</t>
         </is>
       </c>
     </row>
@@ -16137,7 +16137,7 @@
       </c>
       <c r="C920" t="inlineStr">
         <is>
-          <t>18초마다 공격력이 잠시 오른다</t>
+          <t>Briefly increases physical attack every 18 seconds while in battle.</t>
         </is>
       </c>
     </row>
@@ -16290,7 +16290,7 @@
       </c>
       <c r="C929" t="inlineStr">
         <is>
-          <t>잔상</t>
+          <t>Afterimage</t>
         </is>
       </c>
     </row>
@@ -16307,7 +16307,7 @@
       </c>
       <c r="C930" t="inlineStr">
         <is>
-          <t>17초마다 회피율이 잠시 오른다</t>
+          <t>Briefly increases evasion every 17 seconds while in battle.</t>
         </is>
       </c>
     </row>
@@ -16426,7 +16426,7 @@
       </c>
       <c r="C937" t="inlineStr">
         <is>
-          <t>강인함</t>
+          <t>Fortitude</t>
         </is>
       </c>
     </row>
@@ -16443,7 +16443,7 @@
       </c>
       <c r="C938" t="inlineStr">
         <is>
-          <t>최대 체력이 오른다</t>
+          <t>Increases max HP.</t>
         </is>
       </c>
     </row>
@@ -16630,7 +16630,7 @@
       </c>
       <c r="C949" t="inlineStr">
         <is>
-          <t>민첩</t>
+          <t>Agility</t>
         </is>
       </c>
     </row>
@@ -16647,7 +16647,7 @@
       </c>
       <c r="C950" t="inlineStr">
         <is>
-          <t>회피율이 오른다</t>
+          <t>Increases evasion.</t>
         </is>
       </c>
     </row>
@@ -16902,7 +16902,7 @@
       </c>
       <c r="C965" t="inlineStr">
         <is>
-          <t>각인</t>
+          <t>Imprint</t>
         </is>
       </c>
     </row>
@@ -16919,7 +16919,7 @@
       </c>
       <c r="C966" t="inlineStr">
         <is>
-          <t>확정 포획에 필요한 횟수가 줄어든다</t>
+          <t>Reduces the number of attempts needed for a guaranteed capture.</t>
         </is>
       </c>
     </row>
@@ -17004,7 +17004,7 @@
       </c>
       <c r="C971" t="inlineStr">
         <is>
-          <t>연계 감각</t>
+          <t>Combo Instinct</t>
         </is>
       </c>
     </row>
@@ -17016,12 +17016,12 @@
       </c>
       <c r="B972" t="inlineStr">
         <is>
-          <t>콤보 게이지가 더 오래 유지된다</t>
+          <t>콤보 유지 시간이 늘어난다.</t>
         </is>
       </c>
       <c r="C972" t="inlineStr">
         <is>
-          <t>콤보 게이지가 더 오래 유지된다</t>
+          <t>Extends the time before a combo expires.</t>
         </is>
       </c>
     </row>
@@ -33983,6 +33983,465 @@
       <c r="C1851" t="inlineStr">
         <is>
           <t>Found:</t>
+        </is>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" t="inlineStr">
+        <is>
+          <t>ClassAbilityCurrentFormat</t>
+        </is>
+      </c>
+      <c r="B1852" t="inlineStr">
+        <is>
+          <t>현재 {0}단계</t>
+        </is>
+      </c>
+      <c r="C1852" t="inlineStr">
+        <is>
+          <t>Current level {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" t="inlineStr">
+        <is>
+          <t>ClassAbilityAcquisitionFormat</t>
+        </is>
+      </c>
+      <c r="B1853" t="inlineStr">
+        <is>
+          <t>습득 시 {0}단계</t>
+        </is>
+      </c>
+      <c r="C1853" t="inlineStr">
+        <is>
+          <t>Upon learning: level {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1854">
+      <c r="A1854" t="inlineStr">
+        <is>
+          <t>ClassAbilityNextFormat</t>
+        </is>
+      </c>
+      <c r="B1854" t="inlineStr">
+        <is>
+          <t>다음 {0}단계</t>
+        </is>
+      </c>
+      <c r="C1854" t="inlineStr">
+        <is>
+          <t>Next level {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" t="inlineStr">
+        <is>
+          <t>ClassAbilityFlatStatFormat</t>
+        </is>
+      </c>
+      <c r="B1855" t="inlineStr">
+        <is>
+          <t>{0} +{1}</t>
+        </is>
+      </c>
+      <c r="C1855" t="inlineStr">
+        <is>
+          <t>{0} +{1}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1856">
+      <c r="A1856" t="inlineStr">
+        <is>
+          <t>ClassAbilityPercentPointFormat</t>
+        </is>
+      </c>
+      <c r="B1856" t="inlineStr">
+        <is>
+          <t>{0} +{1}%p</t>
+        </is>
+      </c>
+      <c r="C1856" t="inlineStr">
+        <is>
+          <t>{0} +{1} percentage points</t>
+        </is>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" t="inlineStr">
+        <is>
+          <t>ClassAbilityComboFormat</t>
+        </is>
+      </c>
+      <c r="B1857" t="inlineStr">
+        <is>
+          <t>콤보 유지 시간 +{0}%</t>
+        </is>
+      </c>
+      <c r="C1857" t="inlineStr">
+        <is>
+          <t>Combo duration +{0}%</t>
+        </is>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" t="inlineStr">
+        <is>
+          <t>ClassAbilityCaptureFormat</t>
+        </is>
+      </c>
+      <c r="B1858" t="inlineStr">
+        <is>
+          <t>확정 포획에 필요한 실패 횟수 -{0}</t>
+        </is>
+      </c>
+      <c r="C1858" t="inlineStr">
+        <is>
+          <t>Failures needed for a guaranteed catch -{0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" t="inlineStr">
+        <is>
+          <t>ClassAbilityChanceFormat</t>
+        </is>
+      </c>
+      <c r="B1859" t="inlineStr">
+        <is>
+          <t>{0}% 확률로 발동</t>
+        </is>
+      </c>
+      <c r="C1859" t="inlineStr">
+        <is>
+          <t>{0}% chance to activate</t>
+        </is>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" t="inlineStr">
+        <is>
+          <t>ClassAbilityIntervalFormat</t>
+        </is>
+      </c>
+      <c r="B1860" t="inlineStr">
+        <is>
+          <t>{0}, 재사용 대기 {1}초</t>
+        </is>
+      </c>
+      <c r="C1860" t="inlineStr">
+        <is>
+          <t>{0}, cooldown {1}s</t>
+        </is>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" t="inlineStr">
+        <is>
+          <t>ClassAbilityHealFormat</t>
+        </is>
+      </c>
+      <c r="B1861" t="inlineStr">
+        <is>
+          <t>HP {0} 회복</t>
+        </is>
+      </c>
+      <c r="C1861" t="inlineStr">
+        <is>
+          <t>Restore {0} HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="1862">
+      <c r="A1862" t="inlineStr">
+        <is>
+          <t>ClassAbilityDamageFormat</t>
+        </is>
+      </c>
+      <c r="B1862" t="inlineStr">
+        <is>
+          <t>추가 피해 {0}</t>
+        </is>
+      </c>
+      <c r="C1862" t="inlineStr">
+        <is>
+          <t>Deal {0} bonus damage</t>
+        </is>
+      </c>
+    </row>
+    <row r="1863">
+      <c r="A1863" t="inlineStr">
+        <is>
+          <t>ClassAbilityHealRatioFormat</t>
+        </is>
+      </c>
+      <c r="B1863" t="inlineStr">
+        <is>
+          <t>{0}의 {1}%만큼 HP 회복</t>
+        </is>
+      </c>
+      <c r="C1863" t="inlineStr">
+        <is>
+          <t>Restore HP equal to {1}% of {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1864">
+      <c r="A1864" t="inlineStr">
+        <is>
+          <t>ClassAbilityDamageRatioFormat</t>
+        </is>
+      </c>
+      <c r="B1864" t="inlineStr">
+        <is>
+          <t>{0}의 {1}%만큼 추가 피해</t>
+        </is>
+      </c>
+      <c r="C1864" t="inlineStr">
+        <is>
+          <t>Deal bonus damage equal to {1}% of {0}</t>
+        </is>
+      </c>
+    </row>
+    <row r="1865">
+      <c r="A1865" t="inlineStr">
+        <is>
+          <t>ClassAbilityDurationFormat</t>
+        </is>
+      </c>
+      <c r="B1865" t="inlineStr">
+        <is>
+          <t>{0} ({1}초)</t>
+        </is>
+      </c>
+      <c r="C1865" t="inlineStr">
+        <is>
+          <t>{0} ({1}s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1866">
+      <c r="A1866" t="inlineStr">
+        <is>
+          <t>ClassAbilityUntilBattleEndFormat</t>
+        </is>
+      </c>
+      <c r="B1866" t="inlineStr">
+        <is>
+          <t>{0} (전투 종료까지)</t>
+        </is>
+      </c>
+      <c r="C1866" t="inlineStr">
+        <is>
+          <t>{0} (until battle ends)</t>
+        </is>
+      </c>
+    </row>
+    <row r="1867">
+      <c r="A1867" t="inlineStr">
+        <is>
+          <t>ClassAbilityBattleStartText</t>
+        </is>
+      </c>
+      <c r="B1867" t="inlineStr">
+        <is>
+          <t>지역 전투 시작 시</t>
+        </is>
+      </c>
+      <c r="C1867" t="inlineStr">
+        <is>
+          <t>At the start of an area's battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="1868">
+      <c r="A1868" t="inlineStr">
+        <is>
+          <t>ClassAbilityConsecutiveCritFormat</t>
+        </is>
+      </c>
+      <c r="B1868" t="inlineStr">
+        <is>
+          <t>{0}회 연속 치명타 시</t>
+        </is>
+      </c>
+      <c r="C1868" t="inlineStr">
+        <is>
+          <t>After {0} consecutive critical hits</t>
+        </is>
+      </c>
+    </row>
+    <row r="1869">
+      <c r="A1869" t="inlineStr">
+        <is>
+          <t>ClassAbilityConsecutiveEvadeFormat</t>
+        </is>
+      </c>
+      <c r="B1869" t="inlineStr">
+        <is>
+          <t>{0}회 연속 회피 시</t>
+        </is>
+      </c>
+      <c r="C1869" t="inlineStr">
+        <is>
+          <t>After {0} consecutive evades</t>
+        </is>
+      </c>
+    </row>
+    <row r="1870">
+      <c r="A1870" t="inlineStr">
+        <is>
+          <t>ClassAbilityFatalDamageText</t>
+        </is>
+      </c>
+      <c r="B1870" t="inlineStr">
+        <is>
+          <t>치명적인 피해를 받기 직전</t>
+        </is>
+      </c>
+      <c r="C1870" t="inlineStr">
+        <is>
+          <t>Before taking lethal damage</t>
+        </is>
+      </c>
+    </row>
+    <row r="1871">
+      <c r="A1871" t="inlineStr">
+        <is>
+          <t>ClassAbilityInBattleText</t>
+        </is>
+      </c>
+      <c r="B1871" t="inlineStr">
+        <is>
+          <t>전투 중 자동 발동</t>
+        </is>
+      </c>
+      <c r="C1871" t="inlineStr">
+        <is>
+          <t>Activates automatically in battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="1872">
+      <c r="A1872" t="inlineStr">
+        <is>
+          <t>ClassAbilityOutOfBattleText</t>
+        </is>
+      </c>
+      <c r="B1872" t="inlineStr">
+        <is>
+          <t>비전투 중 자동 발동</t>
+        </is>
+      </c>
+      <c r="C1872" t="inlineStr">
+        <is>
+          <t>Activates automatically outside battle</t>
+        </is>
+      </c>
+    </row>
+    <row r="1873">
+      <c r="A1873" t="inlineStr">
+        <is>
+          <t>ClassAbilityAlwaysText</t>
+        </is>
+      </c>
+      <c r="B1873" t="inlineStr">
+        <is>
+          <t>항상 자동 발동</t>
+        </is>
+      </c>
+      <c r="C1873" t="inlineStr">
+        <is>
+          <t>Activates automatically at any time</t>
+        </is>
+      </c>
+    </row>
+    <row r="1874">
+      <c r="A1874" t="inlineStr">
+        <is>
+          <t>ClassAbilityOrText</t>
+        </is>
+      </c>
+      <c r="B1874" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 또는 </t>
+        </is>
+      </c>
+      <c r="C1874" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> or </t>
+        </is>
+      </c>
+    </row>
+    <row r="1875">
+      <c r="A1875" t="inlineStr">
+        <is>
+          <t>ClassAbilityMaxHpText</t>
+        </is>
+      </c>
+      <c r="B1875" t="inlineStr">
+        <is>
+          <t>최대 HP</t>
+        </is>
+      </c>
+      <c r="C1875" t="inlineStr">
+        <is>
+          <t>Max HP</t>
+        </is>
+      </c>
+    </row>
+    <row r="1876">
+      <c r="A1876" t="inlineStr">
+        <is>
+          <t>ClassAbilityDefText</t>
+        </is>
+      </c>
+      <c r="B1876" t="inlineStr">
+        <is>
+          <t>방어력</t>
+        </is>
+      </c>
+      <c r="C1876" t="inlineStr">
+        <is>
+          <t>Defense</t>
+        </is>
+      </c>
+    </row>
+    <row r="1877">
+      <c r="A1877" t="inlineStr">
+        <is>
+          <t>ClassAbilityEvasionText</t>
+        </is>
+      </c>
+      <c r="B1877" t="inlineStr">
+        <is>
+          <t>회피율</t>
+        </is>
+      </c>
+      <c r="C1877" t="inlineStr">
+        <is>
+          <t>Evasion</t>
+        </is>
+      </c>
+    </row>
+    <row r="1878">
+      <c r="A1878" t="inlineStr">
+        <is>
+          <t>ClassAbilityPhysicalAtkText</t>
+        </is>
+      </c>
+      <c r="B1878" t="inlineStr">
+        <is>
+          <t>물리 공격력</t>
+        </is>
+      </c>
+      <c r="C1878" t="inlineStr">
+        <is>
+          <t>Physical attack</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: use the game's own term "Minimon" instead of "minion" in English
UI 라벨은 MINIMON(도감·나의 미니몬)인데 능력 설명 507행은 'minion' 이라 한 화면에 두 이름이 섞였다.
영문 제목도 Minimon Quest — 고유명처럼 복수형 없이 'Minimon'(스토어 문구와 동일).
재현: python _tools/normalize_minimon_term.py --write → Tools/ParseAllLocal (JSON 에 'minion' 0건)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assets/@Resources/Data/Excel/LocalizationData.xlsx
+++ b/Assets/@Resources/Data/Excel/LocalizationData.xlsx
@@ -4930,7 +4930,7 @@
         <is>
           <t>Passive: +30 maximum HP per ability level.
 Manual use: Restore 18% of maximum HP per ability level.
-Cooldown: 18s, shared by minion abilities.
+Cooldown: 18s, shared by Minimon abilities.
 Available temporarily while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -4989,7 +4989,7 @@
         <is>
           <t>Passive: +10 percentage points of attack speed per ability level.
 Manual use: Gain 30 percentage points of attack speed per ability level for 8 seconds.
-Cooldown: 18s, shared by minion abilities.
+Cooldown: 18s, shared by Minimon abilities.
 Available temporarily while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Increases minion catch success rate.</t>
+          <t>Increases Minimon catch success rate.</t>
         </is>
       </c>
     </row>
@@ -16885,7 +16885,7 @@
       </c>
       <c r="C964" t="inlineStr">
         <is>
-          <t>Increases minion catch success rate.</t>
+          <t>Increases Minimon catch success rate.</t>
         </is>
       </c>
     </row>
@@ -16953,7 +16953,7 @@
       </c>
       <c r="C968" t="inlineStr">
         <is>
-          <t>Increases the number of attracted minions you can hold.</t>
+          <t>Increases the number of attracted Minimon you can hold.</t>
         </is>
       </c>
     </row>
@@ -23292,7 +23292,7 @@
       <c r="C1340" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23313,7 +23313,7 @@
       <c r="C1341" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23334,7 +23334,7 @@
       <c r="C1342" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23355,7 +23355,7 @@
       <c r="C1343" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23376,7 +23376,7 @@
       <c r="C1344" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23397,7 +23397,7 @@
       <c r="C1345" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23418,7 +23418,7 @@
       <c r="C1346" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23439,7 +23439,7 @@
       <c r="C1347" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23460,7 +23460,7 @@
       <c r="C1348" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23481,7 +23481,7 @@
       <c r="C1349" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23502,7 +23502,7 @@
       <c r="C1350" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23523,7 +23523,7 @@
       <c r="C1351" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23544,7 +23544,7 @@
       <c r="C1352" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23565,7 +23565,7 @@
       <c r="C1353" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23586,7 +23586,7 @@
       <c r="C1354" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23607,7 +23607,7 @@
       <c r="C1355" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23628,7 +23628,7 @@
       <c r="C1356" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23649,7 +23649,7 @@
       <c r="C1357" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23670,7 +23670,7 @@
       <c r="C1358" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23691,7 +23691,7 @@
       <c r="C1359" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23712,7 +23712,7 @@
       <c r="C1360" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23733,7 +23733,7 @@
       <c r="C1361" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23754,7 +23754,7 @@
       <c r="C1362" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23775,7 +23775,7 @@
       <c r="C1363" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23796,7 +23796,7 @@
       <c r="C1364" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23817,7 +23817,7 @@
       <c r="C1365" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23838,7 +23838,7 @@
       <c r="C1366" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23859,7 +23859,7 @@
       <c r="C1367" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23880,7 +23880,7 @@
       <c r="C1368" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23901,7 +23901,7 @@
       <c r="C1369" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23922,7 +23922,7 @@
       <c r="C1370" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23943,7 +23943,7 @@
       <c r="C1371" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23964,7 +23964,7 @@
       <c r="C1372" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -23985,7 +23985,7 @@
       <c r="C1373" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24006,7 +24006,7 @@
       <c r="C1374" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24027,7 +24027,7 @@
       <c r="C1375" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24048,7 +24048,7 @@
       <c r="C1376" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24069,7 +24069,7 @@
       <c r="C1377" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24090,7 +24090,7 @@
       <c r="C1378" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24111,7 +24111,7 @@
       <c r="C1379" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24132,7 +24132,7 @@
       <c r="C1380" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24153,7 +24153,7 @@
       <c r="C1381" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24174,7 +24174,7 @@
       <c r="C1382" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24195,7 +24195,7 @@
       <c r="C1383" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24216,7 +24216,7 @@
       <c r="C1384" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24237,7 +24237,7 @@
       <c r="C1385" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24258,7 +24258,7 @@
       <c r="C1386" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24279,7 +24279,7 @@
       <c r="C1387" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24300,7 +24300,7 @@
       <c r="C1388" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24321,7 +24321,7 @@
       <c r="C1389" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24342,7 +24342,7 @@
       <c r="C1390" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24363,7 +24363,7 @@
       <c r="C1391" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24384,7 +24384,7 @@
       <c r="C1392" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24405,7 +24405,7 @@
       <c r="C1393" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24426,7 +24426,7 @@
       <c r="C1394" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24447,7 +24447,7 @@
       <c r="C1395" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24468,7 +24468,7 @@
       <c r="C1396" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24489,7 +24489,7 @@
       <c r="C1397" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24510,7 +24510,7 @@
       <c r="C1398" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24531,7 +24531,7 @@
       <c r="C1399" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24552,7 +24552,7 @@
       <c r="C1400" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24573,7 +24573,7 @@
       <c r="C1401" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24594,7 +24594,7 @@
       <c r="C1402" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24615,7 +24615,7 @@
       <c r="C1403" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24636,7 +24636,7 @@
       <c r="C1404" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24657,7 +24657,7 @@
       <c r="C1405" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24678,7 +24678,7 @@
       <c r="C1406" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24699,7 +24699,7 @@
       <c r="C1407" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24720,7 +24720,7 @@
       <c r="C1408" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24741,7 +24741,7 @@
       <c r="C1409" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24762,7 +24762,7 @@
       <c r="C1410" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24783,7 +24783,7 @@
       <c r="C1411" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24804,7 +24804,7 @@
       <c r="C1412" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24825,7 +24825,7 @@
       <c r="C1413" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24846,7 +24846,7 @@
       <c r="C1414" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24867,7 +24867,7 @@
       <c r="C1415" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24888,7 +24888,7 @@
       <c r="C1416" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24909,7 +24909,7 @@
       <c r="C1417" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24930,7 +24930,7 @@
       <c r="C1418" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24951,7 +24951,7 @@
       <c r="C1419" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24972,7 +24972,7 @@
       <c r="C1420" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -24993,7 +24993,7 @@
       <c r="C1421" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25014,7 +25014,7 @@
       <c r="C1422" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25035,7 +25035,7 @@
       <c r="C1423" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25056,7 +25056,7 @@
       <c r="C1424" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25077,7 +25077,7 @@
       <c r="C1425" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25098,7 +25098,7 @@
       <c r="C1426" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25119,7 +25119,7 @@
       <c r="C1427" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25140,7 +25140,7 @@
       <c r="C1428" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25161,7 +25161,7 @@
       <c r="C1429" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25182,7 +25182,7 @@
       <c r="C1430" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25203,7 +25203,7 @@
       <c r="C1431" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25224,7 +25224,7 @@
       <c r="C1432" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25245,7 +25245,7 @@
       <c r="C1433" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25266,7 +25266,7 @@
       <c r="C1434" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25287,7 +25287,7 @@
       <c r="C1435" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25308,7 +25308,7 @@
       <c r="C1436" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25329,7 +25329,7 @@
       <c r="C1437" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25350,7 +25350,7 @@
       <c r="C1438" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25371,7 +25371,7 @@
       <c r="C1439" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25392,7 +25392,7 @@
       <c r="C1440" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25413,7 +25413,7 @@
       <c r="C1441" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25434,7 +25434,7 @@
       <c r="C1442" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25455,7 +25455,7 @@
       <c r="C1443" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25476,7 +25476,7 @@
       <c r="C1444" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25497,7 +25497,7 @@
       <c r="C1445" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25518,7 +25518,7 @@
       <c r="C1446" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25539,7 +25539,7 @@
       <c r="C1447" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25560,7 +25560,7 @@
       <c r="C1448" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25581,7 +25581,7 @@
       <c r="C1449" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25602,7 +25602,7 @@
       <c r="C1450" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25623,7 +25623,7 @@
       <c r="C1451" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25644,7 +25644,7 @@
       <c r="C1452" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25665,7 +25665,7 @@
       <c r="C1453" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25686,7 +25686,7 @@
       <c r="C1454" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25707,7 +25707,7 @@
       <c r="C1455" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25728,7 +25728,7 @@
       <c r="C1456" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25749,7 +25749,7 @@
       <c r="C1457" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25770,7 +25770,7 @@
       <c r="C1458" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25791,7 +25791,7 @@
       <c r="C1459" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25812,7 +25812,7 @@
       <c r="C1460" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25833,7 +25833,7 @@
       <c r="C1461" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25854,7 +25854,7 @@
       <c r="C1462" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25875,7 +25875,7 @@
       <c r="C1463" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25896,7 +25896,7 @@
       <c r="C1464" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25917,7 +25917,7 @@
       <c r="C1465" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25938,7 +25938,7 @@
       <c r="C1466" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25959,7 +25959,7 @@
       <c r="C1467" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -25980,7 +25980,7 @@
       <c r="C1468" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26001,7 +26001,7 @@
       <c r="C1469" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26022,7 +26022,7 @@
       <c r="C1470" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26043,7 +26043,7 @@
       <c r="C1471" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26064,7 +26064,7 @@
       <c r="C1472" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26085,7 +26085,7 @@
       <c r="C1473" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26106,7 +26106,7 @@
       <c r="C1474" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26127,7 +26127,7 @@
       <c r="C1475" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26148,7 +26148,7 @@
       <c r="C1476" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26169,7 +26169,7 @@
       <c r="C1477" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26190,7 +26190,7 @@
       <c r="C1478" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26211,7 +26211,7 @@
       <c r="C1479" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26232,7 +26232,7 @@
       <c r="C1480" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26253,7 +26253,7 @@
       <c r="C1481" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26274,7 +26274,7 @@
       <c r="C1482" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26295,7 +26295,7 @@
       <c r="C1483" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26316,7 +26316,7 @@
       <c r="C1484" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26337,7 +26337,7 @@
       <c r="C1485" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26358,7 +26358,7 @@
       <c r="C1486" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26379,7 +26379,7 @@
       <c r="C1487" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26400,7 +26400,7 @@
       <c r="C1488" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26421,7 +26421,7 @@
       <c r="C1489" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26442,7 +26442,7 @@
       <c r="C1490" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26463,7 +26463,7 @@
       <c r="C1491" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26484,7 +26484,7 @@
       <c r="C1492" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26505,7 +26505,7 @@
       <c r="C1493" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26526,7 +26526,7 @@
       <c r="C1494" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26547,7 +26547,7 @@
       <c r="C1495" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26568,7 +26568,7 @@
       <c r="C1496" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26589,7 +26589,7 @@
       <c r="C1497" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26610,7 +26610,7 @@
       <c r="C1498" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26631,7 +26631,7 @@
       <c r="C1499" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26652,7 +26652,7 @@
       <c r="C1500" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26673,7 +26673,7 @@
       <c r="C1501" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26694,7 +26694,7 @@
       <c r="C1502" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26715,7 +26715,7 @@
       <c r="C1503" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26736,7 +26736,7 @@
       <c r="C1504" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26757,7 +26757,7 @@
       <c r="C1505" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26778,7 +26778,7 @@
       <c r="C1506" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26799,7 +26799,7 @@
       <c r="C1507" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26820,7 +26820,7 @@
       <c r="C1508" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26841,7 +26841,7 @@
       <c r="C1509" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26862,7 +26862,7 @@
       <c r="C1510" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26883,7 +26883,7 @@
       <c r="C1511" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26904,7 +26904,7 @@
       <c r="C1512" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26925,7 +26925,7 @@
       <c r="C1513" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26946,7 +26946,7 @@
       <c r="C1514" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26967,7 +26967,7 @@
       <c r="C1515" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -26988,7 +26988,7 @@
       <c r="C1516" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27009,7 +27009,7 @@
       <c r="C1517" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27030,7 +27030,7 @@
       <c r="C1518" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27051,7 +27051,7 @@
       <c r="C1519" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27072,7 +27072,7 @@
       <c r="C1520" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27093,7 +27093,7 @@
       <c r="C1521" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27114,7 +27114,7 @@
       <c r="C1522" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27135,7 +27135,7 @@
       <c r="C1523" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27156,7 +27156,7 @@
       <c r="C1524" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27177,7 +27177,7 @@
       <c r="C1525" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27198,7 +27198,7 @@
       <c r="C1526" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27219,7 +27219,7 @@
       <c r="C1527" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27240,7 +27240,7 @@
       <c r="C1528" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27261,7 +27261,7 @@
       <c r="C1529" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27282,7 +27282,7 @@
       <c r="C1530" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27303,7 +27303,7 @@
       <c r="C1531" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27324,7 +27324,7 @@
       <c r="C1532" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27345,7 +27345,7 @@
       <c r="C1533" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27366,7 +27366,7 @@
       <c r="C1534" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27387,7 +27387,7 @@
       <c r="C1535" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27408,7 +27408,7 @@
       <c r="C1536" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27429,7 +27429,7 @@
       <c r="C1537" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27450,7 +27450,7 @@
       <c r="C1538" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27471,7 +27471,7 @@
       <c r="C1539" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27492,7 +27492,7 @@
       <c r="C1540" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27513,7 +27513,7 @@
       <c r="C1541" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27534,7 +27534,7 @@
       <c r="C1542" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27555,7 +27555,7 @@
       <c r="C1543" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27576,7 +27576,7 @@
       <c r="C1544" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27597,7 +27597,7 @@
       <c r="C1545" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27618,7 +27618,7 @@
       <c r="C1546" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27639,7 +27639,7 @@
       <c r="C1547" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27660,7 +27660,7 @@
       <c r="C1548" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27681,7 +27681,7 @@
       <c r="C1549" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27702,7 +27702,7 @@
       <c r="C1550" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27723,7 +27723,7 @@
       <c r="C1551" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27744,7 +27744,7 @@
       <c r="C1552" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27765,7 +27765,7 @@
       <c r="C1553" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27786,7 +27786,7 @@
       <c r="C1554" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27807,7 +27807,7 @@
       <c r="C1555" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27828,7 +27828,7 @@
       <c r="C1556" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27849,7 +27849,7 @@
       <c r="C1557" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27870,7 +27870,7 @@
       <c r="C1558" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27891,7 +27891,7 @@
       <c r="C1559" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27912,7 +27912,7 @@
       <c r="C1560" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27933,7 +27933,7 @@
       <c r="C1561" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27954,7 +27954,7 @@
       <c r="C1562" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27975,7 +27975,7 @@
       <c r="C1563" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -27996,7 +27996,7 @@
       <c r="C1564" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28017,7 +28017,7 @@
       <c r="C1565" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28038,7 +28038,7 @@
       <c r="C1566" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28059,7 +28059,7 @@
       <c r="C1567" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28080,7 +28080,7 @@
       <c r="C1568" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28101,7 +28101,7 @@
       <c r="C1569" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28122,7 +28122,7 @@
       <c r="C1570" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28143,7 +28143,7 @@
       <c r="C1571" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28164,7 +28164,7 @@
       <c r="C1572" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28185,7 +28185,7 @@
       <c r="C1573" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28206,7 +28206,7 @@
       <c r="C1574" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28227,7 +28227,7 @@
       <c r="C1575" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28248,7 +28248,7 @@
       <c r="C1576" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28269,7 +28269,7 @@
       <c r="C1577" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28290,7 +28290,7 @@
       <c r="C1578" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28311,7 +28311,7 @@
       <c r="C1579" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28332,7 +28332,7 @@
       <c r="C1580" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28353,7 +28353,7 @@
       <c r="C1581" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28374,7 +28374,7 @@
       <c r="C1582" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28395,7 +28395,7 @@
       <c r="C1583" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28416,7 +28416,7 @@
       <c r="C1584" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28437,7 +28437,7 @@
       <c r="C1585" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28458,7 +28458,7 @@
       <c r="C1586" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28479,7 +28479,7 @@
       <c r="C1587" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28500,7 +28500,7 @@
       <c r="C1588" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28521,7 +28521,7 @@
       <c r="C1589" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28542,7 +28542,7 @@
       <c r="C1590" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28563,7 +28563,7 @@
       <c r="C1591" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28584,7 +28584,7 @@
       <c r="C1592" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28605,7 +28605,7 @@
       <c r="C1593" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28626,7 +28626,7 @@
       <c r="C1594" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28647,7 +28647,7 @@
       <c r="C1595" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28668,7 +28668,7 @@
       <c r="C1596" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28689,7 +28689,7 @@
       <c r="C1597" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28710,7 +28710,7 @@
       <c r="C1598" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28731,7 +28731,7 @@
       <c r="C1599" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28752,7 +28752,7 @@
       <c r="C1600" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28773,7 +28773,7 @@
       <c r="C1601" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28794,7 +28794,7 @@
       <c r="C1602" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28815,7 +28815,7 @@
       <c r="C1603" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28836,7 +28836,7 @@
       <c r="C1604" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28857,7 +28857,7 @@
       <c r="C1605" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28878,7 +28878,7 @@
       <c r="C1606" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28899,7 +28899,7 @@
       <c r="C1607" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28920,7 +28920,7 @@
       <c r="C1608" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28941,7 +28941,7 @@
       <c r="C1609" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28962,7 +28962,7 @@
       <c r="C1610" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -28983,7 +28983,7 @@
       <c r="C1611" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29004,7 +29004,7 @@
       <c r="C1612" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29025,7 +29025,7 @@
       <c r="C1613" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29046,7 +29046,7 @@
       <c r="C1614" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29067,7 +29067,7 @@
       <c r="C1615" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29088,7 +29088,7 @@
       <c r="C1616" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29109,7 +29109,7 @@
       <c r="C1617" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29130,7 +29130,7 @@
       <c r="C1618" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29151,7 +29151,7 @@
       <c r="C1619" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29172,7 +29172,7 @@
       <c r="C1620" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29193,7 +29193,7 @@
       <c r="C1621" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29214,7 +29214,7 @@
       <c r="C1622" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29235,7 +29235,7 @@
       <c r="C1623" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29256,7 +29256,7 @@
       <c r="C1624" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29277,7 +29277,7 @@
       <c r="C1625" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29298,7 +29298,7 @@
       <c r="C1626" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29319,7 +29319,7 @@
       <c r="C1627" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29340,7 +29340,7 @@
       <c r="C1628" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29361,7 +29361,7 @@
       <c r="C1629" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29382,7 +29382,7 @@
       <c r="C1630" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29403,7 +29403,7 @@
       <c r="C1631" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29424,7 +29424,7 @@
       <c r="C1632" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29445,7 +29445,7 @@
       <c r="C1633" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29466,7 +29466,7 @@
       <c r="C1634" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29487,7 +29487,7 @@
       <c r="C1635" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29508,7 +29508,7 @@
       <c r="C1636" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29529,7 +29529,7 @@
       <c r="C1637" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29550,7 +29550,7 @@
       <c r="C1638" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29571,7 +29571,7 @@
       <c r="C1639" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29592,7 +29592,7 @@
       <c r="C1640" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29613,7 +29613,7 @@
       <c r="C1641" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29634,7 +29634,7 @@
       <c r="C1642" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29655,7 +29655,7 @@
       <c r="C1643" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29676,7 +29676,7 @@
       <c r="C1644" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29697,7 +29697,7 @@
       <c r="C1645" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29718,7 +29718,7 @@
       <c r="C1646" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29739,7 +29739,7 @@
       <c r="C1647" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29760,7 +29760,7 @@
       <c r="C1648" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29781,7 +29781,7 @@
       <c r="C1649" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29802,7 +29802,7 @@
       <c r="C1650" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29823,7 +29823,7 @@
       <c r="C1651" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29844,7 +29844,7 @@
       <c r="C1652" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29865,7 +29865,7 @@
       <c r="C1653" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29886,7 +29886,7 @@
       <c r="C1654" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29907,7 +29907,7 @@
       <c r="C1655" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29928,7 +29928,7 @@
       <c r="C1656" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29949,7 +29949,7 @@
       <c r="C1657" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29970,7 +29970,7 @@
       <c r="C1658" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -29991,7 +29991,7 @@
       <c r="C1659" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30012,7 +30012,7 @@
       <c r="C1660" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30033,7 +30033,7 @@
       <c r="C1661" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30054,7 +30054,7 @@
       <c r="C1662" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30075,7 +30075,7 @@
       <c r="C1663" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30096,7 +30096,7 @@
       <c r="C1664" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30117,7 +30117,7 @@
       <c r="C1665" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30138,7 +30138,7 @@
       <c r="C1666" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30159,7 +30159,7 @@
       <c r="C1667" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30180,7 +30180,7 @@
       <c r="C1668" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30201,7 +30201,7 @@
       <c r="C1669" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30222,7 +30222,7 @@
       <c r="C1670" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30243,7 +30243,7 @@
       <c r="C1671" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30264,7 +30264,7 @@
       <c r="C1672" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30285,7 +30285,7 @@
       <c r="C1673" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30306,7 +30306,7 @@
       <c r="C1674" t="inlineStr">
         <is>
           <t>Gain 20 percentage points of accuracy for 8 seconds.
-Cooldown: 14s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 14s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30327,7 +30327,7 @@
       <c r="C1675" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30348,7 +30348,7 @@
       <c r="C1676" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30369,7 +30369,7 @@
       <c r="C1677" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30390,7 +30390,7 @@
       <c r="C1678" t="inlineStr">
         <is>
           <t>Gain 30 percentage points of attack speed for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30411,7 +30411,7 @@
       <c r="C1679" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30432,7 +30432,7 @@
       <c r="C1680" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30453,7 +30453,7 @@
       <c r="C1681" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30474,7 +30474,7 @@
       <c r="C1682" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30495,7 +30495,7 @@
       <c r="C1683" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30516,7 +30516,7 @@
       <c r="C1684" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30537,7 +30537,7 @@
       <c r="C1685" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30558,7 +30558,7 @@
       <c r="C1686" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30579,7 +30579,7 @@
       <c r="C1687" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30600,7 +30600,7 @@
       <c r="C1688" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30621,7 +30621,7 @@
       <c r="C1689" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30642,7 +30642,7 @@
       <c r="C1690" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30663,7 +30663,7 @@
       <c r="C1691" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30684,7 +30684,7 @@
       <c r="C1692" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30705,7 +30705,7 @@
       <c r="C1693" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30726,7 +30726,7 @@
       <c r="C1694" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30747,7 +30747,7 @@
       <c r="C1695" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30768,7 +30768,7 @@
       <c r="C1696" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30789,7 +30789,7 @@
       <c r="C1697" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30810,7 +30810,7 @@
       <c r="C1698" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30831,7 +30831,7 @@
       <c r="C1699" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30852,7 +30852,7 @@
       <c r="C1700" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30873,7 +30873,7 @@
       <c r="C1701" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30894,7 +30894,7 @@
       <c r="C1702" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30915,7 +30915,7 @@
       <c r="C1703" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30936,7 +30936,7 @@
       <c r="C1704" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30957,7 +30957,7 @@
       <c r="C1705" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30978,7 +30978,7 @@
       <c r="C1706" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -30999,7 +30999,7 @@
       <c r="C1707" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31020,7 +31020,7 @@
       <c r="C1708" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31041,7 +31041,7 @@
       <c r="C1709" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31062,7 +31062,7 @@
       <c r="C1710" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31083,7 +31083,7 @@
       <c r="C1711" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31104,7 +31104,7 @@
       <c r="C1712" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31125,7 +31125,7 @@
       <c r="C1713" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31146,7 +31146,7 @@
       <c r="C1714" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31167,7 +31167,7 @@
       <c r="C1715" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31188,7 +31188,7 @@
       <c r="C1716" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31209,7 +31209,7 @@
       <c r="C1717" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31230,7 +31230,7 @@
       <c r="C1718" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31251,7 +31251,7 @@
       <c r="C1719" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31272,7 +31272,7 @@
       <c r="C1720" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31293,7 +31293,7 @@
       <c r="C1721" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31314,7 +31314,7 @@
       <c r="C1722" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31335,7 +31335,7 @@
       <c r="C1723" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31356,7 +31356,7 @@
       <c r="C1724" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31377,7 +31377,7 @@
       <c r="C1725" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31398,7 +31398,7 @@
       <c r="C1726" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31419,7 +31419,7 @@
       <c r="C1727" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31440,7 +31440,7 @@
       <c r="C1728" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31461,7 +31461,7 @@
       <c r="C1729" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31482,7 +31482,7 @@
       <c r="C1730" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31503,7 +31503,7 @@
       <c r="C1731" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31524,7 +31524,7 @@
       <c r="C1732" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31545,7 +31545,7 @@
       <c r="C1733" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31566,7 +31566,7 @@
       <c r="C1734" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31587,7 +31587,7 @@
       <c r="C1735" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31608,7 +31608,7 @@
       <c r="C1736" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31629,7 +31629,7 @@
       <c r="C1737" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31650,7 +31650,7 @@
       <c r="C1738" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31671,7 +31671,7 @@
       <c r="C1739" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31692,7 +31692,7 @@
       <c r="C1740" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31713,7 +31713,7 @@
       <c r="C1741" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31734,7 +31734,7 @@
       <c r="C1742" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31755,7 +31755,7 @@
       <c r="C1743" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31776,7 +31776,7 @@
       <c r="C1744" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31797,7 +31797,7 @@
       <c r="C1745" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31818,7 +31818,7 @@
       <c r="C1746" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31839,7 +31839,7 @@
       <c r="C1747" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31860,7 +31860,7 @@
       <c r="C1748" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31881,7 +31881,7 @@
       <c r="C1749" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31902,7 +31902,7 @@
       <c r="C1750" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31923,7 +31923,7 @@
       <c r="C1751" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31944,7 +31944,7 @@
       <c r="C1752" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31965,7 +31965,7 @@
       <c r="C1753" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -31986,7 +31986,7 @@
       <c r="C1754" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32007,7 +32007,7 @@
       <c r="C1755" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32028,7 +32028,7 @@
       <c r="C1756" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32049,7 +32049,7 @@
       <c r="C1757" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32070,7 +32070,7 @@
       <c r="C1758" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32091,7 +32091,7 @@
       <c r="C1759" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32112,7 +32112,7 @@
       <c r="C1760" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32133,7 +32133,7 @@
       <c r="C1761" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32154,7 +32154,7 @@
       <c r="C1762" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32175,7 +32175,7 @@
       <c r="C1763" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32196,7 +32196,7 @@
       <c r="C1764" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32217,7 +32217,7 @@
       <c r="C1765" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32238,7 +32238,7 @@
       <c r="C1766" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32259,7 +32259,7 @@
       <c r="C1767" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32280,7 +32280,7 @@
       <c r="C1768" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32301,7 +32301,7 @@
       <c r="C1769" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32322,7 +32322,7 @@
       <c r="C1770" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32343,7 +32343,7 @@
       <c r="C1771" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32364,7 +32364,7 @@
       <c r="C1772" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32385,7 +32385,7 @@
       <c r="C1773" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32406,7 +32406,7 @@
       <c r="C1774" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32427,7 +32427,7 @@
       <c r="C1775" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32448,7 +32448,7 @@
       <c r="C1776" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32469,7 +32469,7 @@
       <c r="C1777" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32490,7 +32490,7 @@
       <c r="C1778" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32511,7 +32511,7 @@
       <c r="C1779" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32532,7 +32532,7 @@
       <c r="C1780" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32553,7 +32553,7 @@
       <c r="C1781" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32574,7 +32574,7 @@
       <c r="C1782" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32595,7 +32595,7 @@
       <c r="C1783" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32616,7 +32616,7 @@
       <c r="C1784" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32637,7 +32637,7 @@
       <c r="C1785" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32658,7 +32658,7 @@
       <c r="C1786" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32679,7 +32679,7 @@
       <c r="C1787" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32700,7 +32700,7 @@
       <c r="C1788" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32721,7 +32721,7 @@
       <c r="C1789" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32742,7 +32742,7 @@
       <c r="C1790" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32763,7 +32763,7 @@
       <c r="C1791" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32784,7 +32784,7 @@
       <c r="C1792" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32805,7 +32805,7 @@
       <c r="C1793" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32826,7 +32826,7 @@
       <c r="C1794" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32847,7 +32847,7 @@
       <c r="C1795" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32868,7 +32868,7 @@
       <c r="C1796" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32889,7 +32889,7 @@
       <c r="C1797" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32910,7 +32910,7 @@
       <c r="C1798" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32931,7 +32931,7 @@
       <c r="C1799" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32952,7 +32952,7 @@
       <c r="C1800" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32973,7 +32973,7 @@
       <c r="C1801" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -32994,7 +32994,7 @@
       <c r="C1802" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33015,7 +33015,7 @@
       <c r="C1803" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33036,7 +33036,7 @@
       <c r="C1804" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33057,7 +33057,7 @@
       <c r="C1805" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33078,7 +33078,7 @@
       <c r="C1806" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33099,7 +33099,7 @@
       <c r="C1807" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33120,7 +33120,7 @@
       <c r="C1808" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33141,7 +33141,7 @@
       <c r="C1809" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33162,7 +33162,7 @@
       <c r="C1810" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33183,7 +33183,7 @@
       <c r="C1811" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33204,7 +33204,7 @@
       <c r="C1812" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33225,7 +33225,7 @@
       <c r="C1813" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33246,7 +33246,7 @@
       <c r="C1814" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33267,7 +33267,7 @@
       <c r="C1815" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33288,7 +33288,7 @@
       <c r="C1816" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33309,7 +33309,7 @@
       <c r="C1817" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33330,7 +33330,7 @@
       <c r="C1818" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33351,7 +33351,7 @@
       <c r="C1819" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33372,7 +33372,7 @@
       <c r="C1820" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33393,7 +33393,7 @@
       <c r="C1821" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33414,7 +33414,7 @@
       <c r="C1822" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33435,7 +33435,7 @@
       <c r="C1823" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33456,7 +33456,7 @@
       <c r="C1824" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33477,7 +33477,7 @@
       <c r="C1825" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33498,7 +33498,7 @@
       <c r="C1826" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33519,7 +33519,7 @@
       <c r="C1827" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33540,7 +33540,7 @@
       <c r="C1828" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33561,7 +33561,7 @@
       <c r="C1829" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33582,7 +33582,7 @@
       <c r="C1830" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33603,7 +33603,7 @@
       <c r="C1831" t="inlineStr">
         <is>
           <t>Gain 18 percentage points of evasion for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33624,7 +33624,7 @@
       <c r="C1832" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33645,7 +33645,7 @@
       <c r="C1833" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33666,7 +33666,7 @@
       <c r="C1834" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33687,7 +33687,7 @@
       <c r="C1835" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 180% of physical attack.
-Cooldown: 12s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 12s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33708,7 +33708,7 @@
       <c r="C1836" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33729,7 +33729,7 @@
       <c r="C1837" t="inlineStr">
         <is>
           <t>Restore 18% of maximum HP.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33750,7 +33750,7 @@
       <c r="C1838" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33771,7 +33771,7 @@
       <c r="C1839" t="inlineStr">
         <is>
           <t>Deal guaranteed bonus damage equal to 300% of physical attack.
-Cooldown: 20s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 20s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -33792,7 +33792,7 @@
       <c r="C1840" t="inlineStr">
         <is>
           <t>Gain 25 percentage points of physical resistance for 8 seconds.
-Cooldown: 18s, shared by minion abilities. Effect scales with ability level.
+Cooldown: 18s, shared by Minimon abilities. Effect scales with ability level.
 Available while accompanying. Permanently learned at 100% resonance.</t>
         </is>
       </c>
@@ -35087,7 +35087,7 @@
       </c>
       <c r="C1916" t="inlineStr">
         <is>
-          <t>attracted minion capacity</t>
+          <t>attracted Minimon capacity</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: localize prefab-baked Korean labels left in English mode
영어 모드에서 주요 팝업 13종을 한 프레임씩 열어 한글이 남은 TMP 를 전수 스캔해 찾은 것:
캐릭터창 '능력 상세정보', 가방 제목 '소지품'·'정리', 마물 상세 '100% 동기화 필요'·
'하수인 또는 완벽분석 필요'·'전리품', 미니몬 정보 '미보유', 물약 [정보](같은 이름 노드 여럿).
키 6개 추가(기존 LootText·CharPopupAttributeDetailText 재사용), 재스캔 결과 실제 경로 기준 0건.
fix_english_localization.py 는 'Minimon' 용어 통일을 반영해 다시 돌려도 같은 결과.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assets/@Resources/Data/Excel/LocalizationData.xlsx
+++ b/Assets/@Resources/Data/Excel/LocalizationData.xlsx
@@ -328,7 +328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1946"/>
+  <dimension ref="A1:C1952"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35607,6 +35607,108 @@
         </is>
       </c>
     </row>
+    <row r="1947">
+      <c r="A1947" t="inlineStr">
+        <is>
+          <t>InventoryTitleText</t>
+        </is>
+      </c>
+      <c r="B1947" t="inlineStr">
+        <is>
+          <t>소지품</t>
+        </is>
+      </c>
+      <c r="C1947" t="inlineStr">
+        <is>
+          <t>INVENTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="1948">
+      <c r="A1948" t="inlineStr">
+        <is>
+          <t>InventorySortText</t>
+        </is>
+      </c>
+      <c r="B1948" t="inlineStr">
+        <is>
+          <t>정리</t>
+        </is>
+      </c>
+      <c r="C1948" t="inlineStr">
+        <is>
+          <t>SORT</t>
+        </is>
+      </c>
+    </row>
+    <row r="1949">
+      <c r="A1949" t="inlineStr">
+        <is>
+          <t>MonsterSkillNeedLinkText</t>
+        </is>
+      </c>
+      <c r="B1949" t="inlineStr">
+        <is>
+          <t>100% 동기화 필요</t>
+        </is>
+      </c>
+      <c r="C1949" t="inlineStr">
+        <is>
+          <t>REQUIRES 100% LINK</t>
+        </is>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>MonsterSkillFullLockText</t>
+        </is>
+      </c>
+      <c r="B1950" t="inlineStr">
+        <is>
+          <t>하수인 또는 완벽분석 필요</t>
+        </is>
+      </c>
+      <c r="C1950" t="inlineStr">
+        <is>
+          <t>REQUIRES MINIMON OR FULL LOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>NotOwnedText</t>
+        </is>
+      </c>
+      <c r="B1951" t="inlineStr">
+        <is>
+          <t>미보유</t>
+        </is>
+      </c>
+      <c r="C1951" t="inlineStr">
+        <is>
+          <t>NOT OWNED</t>
+        </is>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" t="inlineStr">
+        <is>
+          <t>InfoBtnText</t>
+        </is>
+      </c>
+      <c r="B1952" t="inlineStr">
+        <is>
+          <t>정보</t>
+        </is>
+      </c>
+      <c r="C1952" t="inlineStr">
+        <is>
+          <t>INFO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: localize alchemy order and potion detail labels in English
2차 영어 전수 스캔(제작·강화·장비상세·상점·구매확인·제작의뢰·물약상세·아이템·포획·설정·크레딧)에서
남은 한국어: 제작의뢰 인사말(코드 하드코딩)과 물약/기술 탭, 물약 상세의 획득처 '연금공방'·[물약개선]·[제작].
기존 키(AlchemyText, CraftText, BtmPotionBtnText, AbilityCodex_BtmText_Skill) 재사용 + 키 2개 추가.
재스캔: 의도된 '한국어' 언어 버튼·크레딧 제목 외 0건(1·2차 합계 팝업 25종).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Assets/@Resources/Data/Excel/LocalizationData.xlsx
+++ b/Assets/@Resources/Data/Excel/LocalizationData.xlsx
@@ -328,7 +328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1952"/>
+  <dimension ref="A1:C1954"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -35709,6 +35709,40 @@
         </is>
       </c>
     </row>
+    <row r="1953">
+      <c r="A1953" t="inlineStr">
+        <is>
+          <t>PotionUpgradeText</t>
+        </is>
+      </c>
+      <c r="B1953" t="inlineStr">
+        <is>
+          <t>물약개선</t>
+        </is>
+      </c>
+      <c r="C1953" t="inlineStr">
+        <is>
+          <t>UPGRADE</t>
+        </is>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" t="inlineStr">
+        <is>
+          <t>CustomOrderGreetingText</t>
+        </is>
+      </c>
+      <c r="B1954" t="inlineStr">
+        <is>
+          <t>"무엇을 만들어드릴까요?"</t>
+        </is>
+      </c>
+      <c r="C1954" t="inlineStr">
+        <is>
+          <t>"What shall I brew for you?"</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>